<commit_message>
Update Indonesia model outputs and analyses
</commit_message>
<xml_diff>
--- a/data/indonesia_model_inputs_public_health_updated_mortality.xlsx
+++ b/data/indonesia_model_inputs_public_health_updated_mortality.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwnetid-my.sharepoint.com/personal/wrgg_uw_edu/Documents/02Work/WorldBank-Indonesia/uw-wb-indonesia-ncd/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="23" documentId="11_5BD1CC8A96289BD2CF13031488BDC7A105240A93" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2EEB4E9C-9BB3-4258-95AB-4891199D7C1A}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="11_5BD1CC8A96289BD2CF13031488BDC7A105240A93" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0B985DDB-2372-4E12-9C09-BDD224550F2C}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -45,6 +45,24 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={B115BCF6-C10A-4345-A98E-EF93B6200499}</author>
+  </authors>
+  <commentList>
+    <comment ref="S2" authorId="0" shapeId="0" xr:uid="{B115BCF6-C10A-4345-A98E-EF93B6200499}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Updated to 61.39% to match the 724K deaths of tobacco analysis</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4548" uniqueCount="1216">
   <si>
@@ -3717,68 +3735,80 @@
       <sz val="11"/>
       <color rgb="FF1F1F1F"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FF9C6500"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF7F6000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FF1F1F1F"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF1F1F1F"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
       <color rgb="FF1F4E78"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF44546A"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="18"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -4448,6 +4478,12 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="William R Garcia" id="{0B877204-B2C5-4430-B652-0328A906551F}" userId="S::wrgg@uw.edu::52698913-8803-44d0-b81a-d207944fdb38" providerId="AD"/>
+</personList>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="PHAssumptionsTable" displayName="PHAssumptionsTable" ref="A1:H37" totalsRowShown="0">
   <tableColumns count="8">
@@ -4645,7 +4681,6 @@
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="PHInterventionCauseMap" displayName="PHInterventionCauseMap" ref="A1:Q62" totalsRowShown="0">
-  <autoFilter ref="A1:Q62" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0400-000001000000}" name="intervention_cause_key"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0400-000002000000}" name="intervention_id"/>
@@ -4961,6 +4996,14 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="S2" dT="2026-08-29T15:08:01.16" personId="{0B877204-B2C5-4430-B652-0328A906551F}" id="{B115BCF6-C10A-4345-A98E-EF93B6200499}">
+    <text>Updated to 61.39% to match the 724K deaths of tobacco analysis</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H26"/>
@@ -12503,7 +12546,7 @@
         <v>269</v>
       </c>
       <c r="N28" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O28" s="8">
         <v>0</v>
@@ -12557,7 +12600,7 @@
         <v>269</v>
       </c>
       <c r="N29" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O29" s="8">
         <v>0</v>
@@ -12611,7 +12654,7 @@
         <v>269</v>
       </c>
       <c r="N30" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O30" s="8">
         <v>0</v>
@@ -12665,7 +12708,7 @@
         <v>269</v>
       </c>
       <c r="N31" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O31" s="8">
         <v>0</v>
@@ -12719,7 +12762,7 @@
         <v>269</v>
       </c>
       <c r="N32" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O32" s="8">
         <v>0</v>
@@ -12773,7 +12816,7 @@
         <v>269</v>
       </c>
       <c r="N33" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O33" s="8">
         <v>0</v>
@@ -12827,7 +12870,7 @@
         <v>269</v>
       </c>
       <c r="N34" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O34" s="8">
         <v>0</v>
@@ -12881,7 +12924,7 @@
         <v>269</v>
       </c>
       <c r="N35" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O35" s="8">
         <v>0</v>
@@ -12935,7 +12978,7 @@
         <v>269</v>
       </c>
       <c r="N36" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O36" s="8">
         <v>0</v>
@@ -12989,7 +13032,7 @@
         <v>269</v>
       </c>
       <c r="N37" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O37" s="8">
         <v>0</v>
@@ -13043,7 +13086,7 @@
         <v>269</v>
       </c>
       <c r="N38" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O38" s="8">
         <v>0</v>
@@ -13097,7 +13140,7 @@
         <v>269</v>
       </c>
       <c r="N39" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O39" s="8">
         <v>0</v>
@@ -13151,7 +13194,7 @@
         <v>269</v>
       </c>
       <c r="N40" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O40" s="8">
         <v>0</v>
@@ -13205,7 +13248,7 @@
         <v>269</v>
       </c>
       <c r="N41" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O41" s="8">
         <v>0</v>
@@ -13259,7 +13302,7 @@
         <v>269</v>
       </c>
       <c r="N42" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O42" s="8">
         <v>0</v>
@@ -13313,7 +13356,7 @@
         <v>269</v>
       </c>
       <c r="N43" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O43" s="8">
         <v>0</v>
@@ -14362,7 +14405,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AB13"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
@@ -14486,11 +14529,11 @@
       </c>
       <c r="F2" s="14">
         <f t="shared" ref="F2:F13" si="0">IF(OR(E2="tax_share_to_price_elasticity",E2="price_elasticity"),S2,X2)</f>
-        <v>0.6139</v>
+        <v>0.38</v>
       </c>
       <c r="G2" s="14">
         <f t="shared" ref="G2:G13" si="1">IF(OR(E2="tax_share_to_price_elasticity",E2="price_elasticity"),T2,Y2)</f>
-        <v>0.75</v>
+        <v>0.47889999999999999</v>
       </c>
       <c r="H2" s="8" t="str">
         <f t="shared" ref="H2:H13" si="2">IF(OR(E2="tax_share_to_price_elasticity",E2="price_elasticity"),U2,"implementation score 0-1")</f>
@@ -14504,7 +14547,7 @@
       </c>
       <c r="K2" s="16">
         <f t="shared" ref="K2:K13" si="3">IF(E2="tax_share_to_price_elasticity",MIN(1,ABS(I2)*AA2),IF(E2="price_elasticity",MIN(1,ABS(I2)*AA2),IF(E2="regulatory_gap_multiplicative",MIN(1,Z2*I2),"")))</f>
-        <v>0.26131199999999999</v>
+        <v>9.1099597006332717E-2</v>
       </c>
       <c r="L2" s="8" t="s">
         <v>377</v>
@@ -14529,10 +14572,10 @@
         <v>380</v>
       </c>
       <c r="S2" s="10">
-        <v>0.6139</v>
+        <v>0.38</v>
       </c>
       <c r="T2" s="10">
-        <v>0.75</v>
+        <v>0.47889999999999999</v>
       </c>
       <c r="U2" s="8" t="s">
         <v>381</v>
@@ -14557,11 +14600,11 @@
       </c>
       <c r="AA2" s="14">
         <f t="shared" ref="AA2:AA13" si="6">IF(E2="tax_share_to_price_elasticity",IF(OR(COUNT(S2,T2)&lt;2,T2&gt;=1),"",MAX(0,(1-S2)/(1-T2)-1)),IF(E2="price_elasticity",IF(COUNT(S2,T2)&lt;2,"",MAX(0,T2-S2)),0))</f>
-        <v>0.5444</v>
+        <v>0.1897908270965265</v>
       </c>
       <c r="AB2" s="14">
-        <f t="shared" ref="AB2:AB13" si="7">IF(OR(E2="tax_share_to_price_elasticity",E2="price_elasticity"),IF(COUNT(S2,T2)&lt;2,"",T2-S2),0)</f>
-        <v>0.1361</v>
+        <f>IF(OR(E2="tax_share_to_price_elasticity",E2="price_elasticity"),IF(COUNT(S2,T2)&lt;2,"",T2-S2),0)</f>
+        <v>9.8899999999999988E-2</v>
       </c>
     </row>
     <row r="3" spans="1:28" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -14656,7 +14699,7 @@
         <v>0.25</v>
       </c>
       <c r="AB3" s="14">
-        <f t="shared" si="7"/>
+        <f t="shared" ref="AB3:AB13" si="7">IF(OR(E3="tax_share_to_price_elasticity",E3="price_elasticity"),IF(COUNT(S3,T3)&lt;2,"",T3-S3),0)</f>
         <v>0.25</v>
       </c>
     </row>
@@ -15598,9 +15641,10 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
 </file>
@@ -15707,29 +15751,31 @@
       <c r="H2" s="18" t="s">
         <v>452</v>
       </c>
-      <c r="I2" s="17"/>
+      <c r="I2" s="17">
+        <v>9.5000000000000001E-2</v>
+      </c>
       <c r="J2" s="16">
         <f>SUMIF(Policy_Levers!$B$2:$B$13,B2,Policy_Levers!$K$2:$K$13)</f>
-        <v>0.26131199999999999</v>
+        <v>9.1099597006332717E-2</v>
       </c>
       <c r="K2" s="16">
         <f t="shared" ref="K2:K13" si="0">IF(ISBLANK(I2),J2,I2)</f>
-        <v>0.26131199999999999</v>
+        <v>9.5000000000000001E-2</v>
       </c>
       <c r="L2" s="18">
         <v>0</v>
       </c>
       <c r="M2" s="18">
         <f t="shared" ref="M2:M13" si="1">IF(OR(ISBLANK(G2),ISBLANK(K2)),"",IF(H2="relative",MAX(L2,G2*(1-K2)),IF(H2="absolute",MAX(L2,G2-K2),IF(H2="target",MAX(L2,K2),""))))</f>
-        <v>0.223822464</v>
+        <v>0.27421499999999999</v>
       </c>
       <c r="N2" s="18">
         <f t="shared" ref="N2:N13" si="2">IF(ISBLANK(M2),"",G2-M2)</f>
-        <v>7.9177535999999993E-2</v>
+        <v>2.8785000000000005E-2</v>
       </c>
       <c r="O2" s="16">
         <f t="shared" ref="O2:O13" si="3">IF(OR(ISBLANK(G2),G2=0,ISBLANK(N2)),"",N2/G2)</f>
-        <v>0.26131199999999999</v>
+        <v>9.5000000000000015E-2</v>
       </c>
       <c r="P2" s="8">
         <f>Assumptions!$B$4</f>
@@ -24493,15 +24539,15 @@
       </c>
       <c r="H2" s="18">
         <f>SUMIF(Exposure_Targets!$B$2:$B$13,INDEX(Intervention_Cause_Map!$B$2:$B$62,MATCH(A2,Intervention_Cause_Map!$A$2:$A$62,0)),Exposure_Targets!$M$2:$M$13)</f>
-        <v>0.223822464</v>
+        <v>0.27421499999999999</v>
       </c>
       <c r="I2" s="18">
         <f t="shared" ref="I2:I33" si="0">G2-H2</f>
-        <v>7.9177535999999993E-2</v>
+        <v>2.8785000000000005E-2</v>
       </c>
       <c r="J2" s="18">
         <f t="shared" ref="J2:J33" si="1">IF(G2=0,0,I2/G2)</f>
-        <v>0.26131199999999999</v>
+        <v>9.5000000000000015E-2</v>
       </c>
       <c r="K2" s="18" t="str">
         <f>INDEX(Effect_Parameters!$F$2:$F$62,MATCH(A2,Effect_Parameters!$B$2:$B$62,0))</f>
@@ -24521,7 +24567,7 @@
       </c>
       <c r="O2" s="18">
         <f>IF(K2="direct_smoking_prevalence_shift_rr",IF(OR(ISBLANK(G2),ISBLANK(H2),ISBLANK(L2)),"",1-(1+H2*(L2-1))/(1+G2*(L2-1))),IF(K2="tobacco_mortality_prevalence_shift_rr",IF(OR(ISBLANK(G2),ISBLANK(H2),ISBLANK(L2)),"",1-(1+H2*(L2-1)+(G2-H2)*(1-SUMIF(Assumptions!$A$2:$A$37,"tobacco_vascular_erd_ge10_pooled",Assumptions!$B$2:$B$37))*(L2-1))/(1+G2*(L2-1))),IF(K2="direct_loglinear_rr_per_unit_reduction",IF(OR(ISBLANK(L2),ISBLANK(I2)),"",1-1/(L2^I2)),IF(K2="tfa_attributable_ihd_PAF_x_regulatory_gap",IF(ISBLANK(M2),"",M2*SUMIF(Policy_Levers!$B$2:$B$13,INDEX(Intervention_Cause_Map!$B$2:$B$62,MATCH(A2,Intervention_Cause_Map!$A$2:$A$62,0)),Policy_Levers!$Z$2:$Z$13)),""))))</f>
-        <v>4.0198444406836953E-2</v>
+        <v>1.4614147909967845E-2</v>
       </c>
       <c r="P2" s="8" t="str">
         <f>INDEX(Intervention_Cause_Map!$J$2:$J$62,MATCH(A2,Intervention_Cause_Map!$A$2:$A$62,0))</f>
@@ -24565,15 +24611,15 @@
       </c>
       <c r="H3" s="18">
         <f>SUMIF(Exposure_Targets!$B$2:$B$13,INDEX(Intervention_Cause_Map!$B$2:$B$62,MATCH(A3,Intervention_Cause_Map!$A$2:$A$62,0)),Exposure_Targets!$M$2:$M$13)</f>
-        <v>0.223822464</v>
+        <v>0.27421499999999999</v>
       </c>
       <c r="I3" s="18">
         <f t="shared" si="0"/>
-        <v>7.9177535999999993E-2</v>
+        <v>2.8785000000000005E-2</v>
       </c>
       <c r="J3" s="18">
         <f t="shared" si="1"/>
-        <v>0.26131199999999999</v>
+        <v>9.5000000000000015E-2</v>
       </c>
       <c r="K3" s="18" t="str">
         <f>INDEX(Effect_Parameters!$F$2:$F$62,MATCH(A3,Effect_Parameters!$B$2:$B$62,0))</f>
@@ -24593,7 +24639,7 @@
       </c>
       <c r="O3" s="18">
         <f>IF(K3="direct_smoking_prevalence_shift_rr",IF(OR(ISBLANK(G3),ISBLANK(H3),ISBLANK(L3)),"",1-(1+H3*(L3-1))/(1+G3*(L3-1))),IF(K3="tobacco_mortality_prevalence_shift_rr",IF(OR(ISBLANK(G3),ISBLANK(H3),ISBLANK(L3)),"",1-(1+H3*(L3-1)+(G3-H3)*(1-SUMIF(Assumptions!$A$2:$A$37,"tobacco_vascular_erd_ge10_pooled",Assumptions!$B$2:$B$37))*(L3-1))/(1+G3*(L3-1))),IF(K3="direct_loglinear_rr_per_unit_reduction",IF(OR(ISBLANK(L3),ISBLANK(I3)),"",1-1/(L3^I3)),IF(K3="tfa_attributable_ihd_PAF_x_regulatory_gap",IF(ISBLANK(M3),"",M3*SUMIF(Policy_Levers!$B$2:$B$13,INDEX(Intervention_Cause_Map!$B$2:$B$62,MATCH(A3,Intervention_Cause_Map!$A$2:$A$62,0)),Policy_Levers!$Z$2:$Z$13)),""))))</f>
-        <v>2.6980884624352219E-2</v>
+        <v>9.8089029180192799E-3</v>
       </c>
       <c r="P3" s="8" t="str">
         <f>INDEX(Intervention_Cause_Map!$J$2:$J$62,MATCH(A3,Intervention_Cause_Map!$A$2:$A$62,0))</f>
@@ -24637,15 +24683,15 @@
       </c>
       <c r="H4" s="18">
         <f>SUMIF(Exposure_Targets!$B$2:$B$13,INDEX(Intervention_Cause_Map!$B$2:$B$62,MATCH(A4,Intervention_Cause_Map!$A$2:$A$62,0)),Exposure_Targets!$M$2:$M$13)</f>
-        <v>0.223822464</v>
+        <v>0.27421499999999999</v>
       </c>
       <c r="I4" s="18">
         <f t="shared" si="0"/>
-        <v>7.9177535999999993E-2</v>
+        <v>2.8785000000000005E-2</v>
       </c>
       <c r="J4" s="18">
         <f t="shared" si="1"/>
-        <v>0.26131199999999999</v>
+        <v>9.5000000000000015E-2</v>
       </c>
       <c r="K4" s="18" t="str">
         <f>INDEX(Effect_Parameters!$F$2:$F$62,MATCH(A4,Effect_Parameters!$B$2:$B$62,0))</f>
@@ -24665,7 +24711,7 @@
       </c>
       <c r="O4" s="18">
         <f>IF(K4="direct_smoking_prevalence_shift_rr",IF(OR(ISBLANK(G4),ISBLANK(H4),ISBLANK(L4)),"",1-(1+H4*(L4-1))/(1+G4*(L4-1))),IF(K4="tobacco_mortality_prevalence_shift_rr",IF(OR(ISBLANK(G4),ISBLANK(H4),ISBLANK(L4)),"",1-(1+H4*(L4-1)+(G4-H4)*(1-SUMIF(Assumptions!$A$2:$A$37,"tobacco_vascular_erd_ge10_pooled",Assumptions!$B$2:$B$37))*(L4-1))/(1+G4*(L4-1))),IF(K4="direct_loglinear_rr_per_unit_reduction",IF(OR(ISBLANK(L4),ISBLANK(I4)),"",1-1/(L4^I4)),IF(K4="tfa_attributable_ihd_PAF_x_regulatory_gap",IF(ISBLANK(M4),"",M4*SUMIF(Policy_Levers!$B$2:$B$13,INDEX(Intervention_Cause_Map!$B$2:$B$62,MATCH(A4,Intervention_Cause_Map!$A$2:$A$62,0)),Policy_Levers!$Z$2:$Z$13)),""))))</f>
-        <v>1.4224809553977424E-2</v>
+        <v>5.1714307327174192E-3</v>
       </c>
       <c r="P4" s="8" t="str">
         <f>INDEX(Intervention_Cause_Map!$J$2:$J$62,MATCH(A4,Intervention_Cause_Map!$A$2:$A$62,0))</f>
@@ -24709,15 +24755,15 @@
       </c>
       <c r="H5" s="18">
         <f>SUMIF(Exposure_Targets!$B$2:$B$13,INDEX(Intervention_Cause_Map!$B$2:$B$62,MATCH(A5,Intervention_Cause_Map!$A$2:$A$62,0)),Exposure_Targets!$M$2:$M$13)</f>
-        <v>0.223822464</v>
+        <v>0.27421499999999999</v>
       </c>
       <c r="I5" s="18">
         <f t="shared" si="0"/>
-        <v>7.9177535999999993E-2</v>
+        <v>2.8785000000000005E-2</v>
       </c>
       <c r="J5" s="18">
         <f t="shared" si="1"/>
-        <v>0.26131199999999999</v>
+        <v>9.5000000000000015E-2</v>
       </c>
       <c r="K5" s="18" t="str">
         <f>INDEX(Effect_Parameters!$F$2:$F$62,MATCH(A5,Effect_Parameters!$B$2:$B$62,0))</f>
@@ -24737,7 +24783,7 @@
       </c>
       <c r="O5" s="18">
         <f>IF(K5="direct_smoking_prevalence_shift_rr",IF(OR(ISBLANK(G5),ISBLANK(H5),ISBLANK(L5)),"",1-(1+H5*(L5-1))/(1+G5*(L5-1))),IF(K5="tobacco_mortality_prevalence_shift_rr",IF(OR(ISBLANK(G5),ISBLANK(H5),ISBLANK(L5)),"",1-(1+H5*(L5-1)+(G5-H5)*(1-SUMIF(Assumptions!$A$2:$A$37,"tobacco_vascular_erd_ge10_pooled",Assumptions!$B$2:$B$37))*(L5-1))/(1+G5*(L5-1))),IF(K5="direct_loglinear_rr_per_unit_reduction",IF(OR(ISBLANK(L5),ISBLANK(I5)),"",1-1/(L5^I5)),IF(K5="tfa_attributable_ihd_PAF_x_regulatory_gap",IF(ISBLANK(M5),"",M5*SUMIF(Policy_Levers!$B$2:$B$13,INDEX(Intervention_Cause_Map!$B$2:$B$62,MATCH(A5,Intervention_Cause_Map!$A$2:$A$62,0)),Policy_Levers!$Z$2:$Z$13)),""))))</f>
-        <v>2.6342437636564742E-2</v>
+        <v>9.5767954608806383E-3</v>
       </c>
       <c r="P5" s="8" t="str">
         <f>INDEX(Intervention_Cause_Map!$J$2:$J$62,MATCH(A5,Intervention_Cause_Map!$A$2:$A$62,0))</f>
@@ -26409,7 +26455,7 @@
       </c>
       <c r="S28" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A28)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A28,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E28="sick",F28="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="29" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26481,7 +26527,7 @@
       </c>
       <c r="S29" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A29)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A29,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E29="sick",F29="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="30" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26553,7 +26599,7 @@
       </c>
       <c r="S30" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A30)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A30,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E30="sick",F30="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="31" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26625,7 +26671,7 @@
       </c>
       <c r="S31" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A31)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A31,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E31="sick",F31="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="32" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26697,7 +26743,7 @@
       </c>
       <c r="S32" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A32)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A32,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E32="sick",F32="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="33" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26769,7 +26815,7 @@
       </c>
       <c r="S33" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A33)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A33,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E33="sick",F33="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="34" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26841,7 +26887,7 @@
       </c>
       <c r="S34" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A34)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A34,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E34="sick",F34="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="35" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26913,7 +26959,7 @@
       </c>
       <c r="S35" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A35)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A35,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E35="sick",F35="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="36" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -26985,7 +27031,7 @@
       </c>
       <c r="S36" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A36)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A36,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E36="sick",F36="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="37" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -27057,7 +27103,7 @@
       </c>
       <c r="S37" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A37)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A37,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E37="sick",F37="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="38" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -27129,7 +27175,7 @@
       </c>
       <c r="S38" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A38)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A38,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E38="sick",F38="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="39" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -27201,7 +27247,7 @@
       </c>
       <c r="S39" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A39)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A39,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E39="sick",F39="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="40" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -27273,7 +27319,7 @@
       </c>
       <c r="S40" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A40)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A40,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E40="sick",F40="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="41" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -27345,7 +27391,7 @@
       </c>
       <c r="S41" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A41)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A41,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E41="sick",F41="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="42" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -27417,7 +27463,7 @@
       </c>
       <c r="S42" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A42)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A42,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E42="sick",F42="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="43" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -27489,7 +27535,7 @@
       </c>
       <c r="S43" s="8" t="str">
         <f>IF(COUNTIF(Effect_Parameters!$B$2:$B$62,A43)&lt;&gt;1,"LINK ERROR",IF(INDEX(Intervention_Cause_Map!$N$2:$N$62,MATCH(A43,Intervention_Cause_Map!$A$2:$A$62,0))=0,"EXPLORATORY - DISABLED",IF(AND(E43="sick",F43="dead"),"R UPDATE REQUIRED","READY FOR MODEL")))</f>
-        <v>READY FOR MODEL</v>
+        <v>EXPLORATORY - DISABLED</v>
       </c>
     </row>
     <row r="44" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -27949,15 +27995,15 @@
       </c>
       <c r="H50" s="19">
         <f>SUMIF(Exposure_Targets!$B$2:$B$13,INDEX(Intervention_Cause_Map!$B$2:$B$62,MATCH(A50,Intervention_Cause_Map!$A$2:$A$62,0)),Exposure_Targets!$M$2:$M$13)</f>
-        <v>0.223822464</v>
+        <v>0.27421499999999999</v>
       </c>
       <c r="I50" s="19">
         <f t="shared" si="2"/>
-        <v>7.9177535999999993E-2</v>
+        <v>2.8785000000000005E-2</v>
       </c>
       <c r="J50" s="19">
         <f>IF(G50=0,0,I50/G50)</f>
-        <v>0.26131199999999999</v>
+        <v>9.5000000000000015E-2</v>
       </c>
       <c r="K50" s="19" t="str">
         <f>INDEX(Effect_Parameters!$F$2:$F$62,MATCH(A50,Effect_Parameters!$B$2:$B$62,0))</f>
@@ -27977,7 +28023,7 @@
       </c>
       <c r="O50" s="19">
         <f>IF(K50="direct_smoking_prevalence_shift_rr",IF(OR(ISBLANK(G50),ISBLANK(H50),ISBLANK(L50)),"",1-(1+H50*(L50-1))/(1+G50*(L50-1))),IF(K50="tobacco_mortality_prevalence_shift_rr",IF(OR(ISBLANK(G50),ISBLANK(H50),ISBLANK(L50)),"",1-(1+H50*(L50-1)+(G50-H50)*(1-SUMIF(Assumptions!$A$2:$A$37,"tobacco_vascular_erd_ge10_pooled",Assumptions!$B$2:$B$37))*(L50-1))/(1+G50*(L50-1))),IF(K50="direct_loglinear_rr_per_unit_reduction",IF(OR(ISBLANK(L50),ISBLANK(I50)),"",1-1/(L50^I50)),IF(K50="tfa_attributable_ihd_PAF_x_regulatory_gap",IF(ISBLANK(M50),"",M50*SUMIF(Policy_Levers!$B$2:$B$13,INDEX(Intervention_Cause_Map!$B$2:$B$62,MATCH(A50,Intervention_Cause_Map!$A$2:$A$62,0)),Policy_Levers!$Z$2:$Z$13)),""))))</f>
-        <v>8.8865198405977508E-2</v>
+        <v>3.2306950498132037E-2</v>
       </c>
       <c r="P50" s="11" t="str">
         <f>INDEX(Intervention_Cause_Map!$J$2:$J$62,MATCH(A50,Intervention_Cause_Map!$A$2:$A$62,0))</f>
@@ -28021,15 +28067,15 @@
       </c>
       <c r="H51" s="19">
         <f>SUMIF(Exposure_Targets!$B$2:$B$13,INDEX(Intervention_Cause_Map!$B$2:$B$62,MATCH(A51,Intervention_Cause_Map!$A$2:$A$62,0)),Exposure_Targets!$M$2:$M$13)</f>
-        <v>0.223822464</v>
+        <v>0.27421499999999999</v>
       </c>
       <c r="I51" s="19">
         <f t="shared" si="2"/>
-        <v>7.9177535999999993E-2</v>
+        <v>2.8785000000000005E-2</v>
       </c>
       <c r="J51" s="19">
         <f t="shared" si="3"/>
-        <v>0.26131199999999999</v>
+        <v>9.5000000000000015E-2</v>
       </c>
       <c r="K51" s="19" t="str">
         <f>INDEX(Effect_Parameters!$F$2:$F$62,MATCH(A51,Effect_Parameters!$B$2:$B$62,0))</f>
@@ -28049,7 +28095,7 @@
       </c>
       <c r="O51" s="19">
         <f>IF(K51="direct_smoking_prevalence_shift_rr",IF(OR(ISBLANK(G51),ISBLANK(H51),ISBLANK(L51)),"",1-(1+H51*(L51-1))/(1+G51*(L51-1))),IF(K51="tobacco_mortality_prevalence_shift_rr",IF(OR(ISBLANK(G51),ISBLANK(H51),ISBLANK(L51)),"",1-(1+H51*(L51-1)+(G51-H51)*(1-SUMIF(Assumptions!$A$2:$A$37,"tobacco_vascular_erd_ge10_pooled",Assumptions!$B$2:$B$37))*(L51-1))/(1+G51*(L51-1))),IF(K51="direct_loglinear_rr_per_unit_reduction",IF(OR(ISBLANK(L51),ISBLANK(I51)),"",1-1/(L51^I51)),IF(K51="tfa_attributable_ihd_PAF_x_regulatory_gap",IF(ISBLANK(M51),"",M51*SUMIF(Policy_Levers!$B$2:$B$13,INDEX(Intervention_Cause_Map!$B$2:$B$62,MATCH(A51,Intervention_Cause_Map!$A$2:$A$62,0)),Policy_Levers!$Z$2:$Z$13)),""))))</f>
-        <v>8.8865198405977508E-2</v>
+        <v>3.2306950498132037E-2</v>
       </c>
       <c r="P51" s="11" t="str">
         <f>INDEX(Intervention_Cause_Map!$J$2:$J$62,MATCH(A51,Intervention_Cause_Map!$A$2:$A$62,0))</f>
@@ -28093,15 +28139,15 @@
       </c>
       <c r="H52" s="19">
         <f>SUMIF(Exposure_Targets!$B$2:$B$13,INDEX(Intervention_Cause_Map!$B$2:$B$62,MATCH(A52,Intervention_Cause_Map!$A$2:$A$62,0)),Exposure_Targets!$M$2:$M$13)</f>
-        <v>0.223822464</v>
+        <v>0.27421499999999999</v>
       </c>
       <c r="I52" s="19">
         <f t="shared" si="2"/>
-        <v>7.9177535999999993E-2</v>
+        <v>2.8785000000000005E-2</v>
       </c>
       <c r="J52" s="19">
         <f t="shared" si="3"/>
-        <v>0.26131199999999999</v>
+        <v>9.5000000000000015E-2</v>
       </c>
       <c r="K52" s="19" t="str">
         <f>INDEX(Effect_Parameters!$F$2:$F$62,MATCH(A52,Effect_Parameters!$B$2:$B$62,0))</f>
@@ -28121,7 +28167,7 @@
       </c>
       <c r="O52" s="19">
         <f>IF(K52="direct_smoking_prevalence_shift_rr",IF(OR(ISBLANK(G52),ISBLANK(H52),ISBLANK(L52)),"",1-(1+H52*(L52-1))/(1+G52*(L52-1))),IF(K52="tobacco_mortality_prevalence_shift_rr",IF(OR(ISBLANK(G52),ISBLANK(H52),ISBLANK(L52)),"",1-(1+H52*(L52-1)+(G52-H52)*(1-SUMIF(Assumptions!$A$2:$A$37,"tobacco_vascular_erd_ge10_pooled",Assumptions!$B$2:$B$37))*(L52-1))/(1+G52*(L52-1))),IF(K52="direct_loglinear_rr_per_unit_reduction",IF(OR(ISBLANK(L52),ISBLANK(I52)),"",1-1/(L52^I52)),IF(K52="tfa_attributable_ihd_PAF_x_regulatory_gap",IF(ISBLANK(M52),"",M52*SUMIF(Policy_Levers!$B$2:$B$13,INDEX(Intervention_Cause_Map!$B$2:$B$62,MATCH(A52,Intervention_Cause_Map!$A$2:$A$62,0)),Policy_Levers!$Z$2:$Z$13)),""))))</f>
-        <v>8.8865198405977508E-2</v>
+        <v>3.2306950498132037E-2</v>
       </c>
       <c r="P52" s="11" t="str">
         <f>INDEX(Intervention_Cause_Map!$J$2:$J$62,MATCH(A52,Intervention_Cause_Map!$A$2:$A$62,0))</f>
@@ -28878,4 +28924,10 @@
     <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{f6b6dd5b-f02f-441a-99a0-162ac5060bd2}" enabled="0" method="" siteId="{f6b6dd5b-f02f-441a-99a0-162ac5060bd2}" removed="1"/>
+</clbl:labelList>
 </file>
</xml_diff>